<commit_message>
filled metadata as example
</commit_message>
<xml_diff>
--- a/examples/hodgskiss_belchers_context.xlsx
+++ b/examples/hodgskiss_belchers_context.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/unafarrell/Dropbox/Database/Templates/git/sgp-context-template/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66325E97-2AED-A848-B21F-7486169A0AAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAAE79A5-E01D-894A-8B78-E9B31364DF48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1580" yWindow="600" windowWidth="32760" windowHeight="18640" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3260" yWindow="1680" windowWidth="32760" windowHeight="18640" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata + Guide" sheetId="8" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1684" uniqueCount="630">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1686" uniqueCount="631">
   <si>
     <t>lith_comp</t>
   </si>
@@ -2165,6 +2165,9 @@
   </si>
   <si>
     <t>Department of Earth and Environmental Sciences, University of Ottawa</t>
+  </si>
+  <si>
+    <t>New version of this context sheet, to serve as an example.</t>
   </si>
 </sst>
 </file>
@@ -2574,7 +2577,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2680,21 +2683,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="201" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -2712,6 +2700,22 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="202">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -3349,10 +3353,10 @@
       </c>
     </row>
     <row r="7" spans="1:4" s="8" customFormat="1" ht="175" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="53" t="s">
+      <c r="A7" s="61" t="s">
         <v>513</v>
       </c>
-      <c r="B7" s="53"/>
+      <c r="B7" s="61"/>
       <c r="C7" s="26"/>
       <c r="D7" s="26"/>
     </row>
@@ -3370,16 +3374,25 @@
       <c r="A10" s="41" t="s">
         <v>510</v>
       </c>
+      <c r="B10" t="s">
+        <v>536</v>
+      </c>
     </row>
     <row r="11" spans="1:4" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="41" t="s">
         <v>508</v>
       </c>
+      <c r="B11" s="65">
+        <v>43815</v>
+      </c>
     </row>
     <row r="12" spans="1:4" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="41" t="s">
         <v>506</v>
       </c>
+      <c r="B12" t="s">
+        <v>630</v>
+      </c>
     </row>
     <row r="13" spans="1:4" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="41"/>
@@ -3391,10 +3404,10 @@
       <c r="B14" s="40"/>
     </row>
     <row r="15" spans="1:4" s="8" customFormat="1" ht="217" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="53" t="s">
+      <c r="A15" s="61" t="s">
         <v>511</v>
       </c>
-      <c r="B15" s="53"/>
+      <c r="B15" s="61"/>
       <c r="C15" s="26"/>
       <c r="D15" s="26"/>
     </row>
@@ -3801,10 +3814,10 @@
       <c r="F3" t="s">
         <v>523</v>
       </c>
-      <c r="G3" s="58">
+      <c r="G3" s="53">
         <v>56.165869999999998</v>
       </c>
-      <c r="H3" s="58">
+      <c r="H3" s="53">
         <v>-78.901403999999999</v>
       </c>
       <c r="I3" t="s">
@@ -3848,10 +3861,10 @@
       <c r="F4" t="s">
         <v>524</v>
       </c>
-      <c r="G4" s="58">
+      <c r="G4" s="53">
         <v>56.1877</v>
       </c>
-      <c r="H4" s="58">
+      <c r="H4" s="53">
         <v>-78.677285999999995</v>
       </c>
       <c r="I4" t="s">
@@ -3895,10 +3908,10 @@
       <c r="F5" t="s">
         <v>525</v>
       </c>
-      <c r="G5" s="58">
+      <c r="G5" s="53">
         <v>56.288739999999997</v>
       </c>
-      <c r="H5" s="58">
+      <c r="H5" s="53">
         <v>-78.967904000000004</v>
       </c>
       <c r="I5" t="s">
@@ -3942,10 +3955,10 @@
       <c r="F6" t="s">
         <v>526</v>
       </c>
-      <c r="G6" s="58">
+      <c r="G6" s="53">
         <v>56.246339999999996</v>
       </c>
-      <c r="H6" s="58">
+      <c r="H6" s="53">
         <v>-78.686890000000005</v>
       </c>
       <c r="I6" t="s">
@@ -3989,10 +4002,10 @@
       <c r="F7" t="s">
         <v>527</v>
       </c>
-      <c r="G7" s="58">
+      <c r="G7" s="53">
         <v>56.189129999999999</v>
       </c>
-      <c r="H7" s="58">
+      <c r="H7" s="53">
         <v>-78.671809999999994</v>
       </c>
       <c r="I7" t="s">
@@ -4036,10 +4049,10 @@
       <c r="F8" t="s">
         <v>528</v>
       </c>
-      <c r="G8" s="58">
+      <c r="G8" s="53">
         <v>56.187309999999997</v>
       </c>
-      <c r="H8" s="58">
+      <c r="H8" s="53">
         <v>-78.666899999999998</v>
       </c>
       <c r="I8" t="s">
@@ -4083,10 +4096,10 @@
       <c r="F9" t="s">
         <v>529</v>
       </c>
-      <c r="G9" s="58">
+      <c r="G9" s="53">
         <v>56.08276</v>
       </c>
-      <c r="H9" s="58">
+      <c r="H9" s="53">
         <v>-78.835710000000006</v>
       </c>
       <c r="I9" t="s">
@@ -4209,10 +4222,10 @@
       <c r="R1" s="35"/>
       <c r="S1" s="35"/>
       <c r="T1" s="35"/>
-      <c r="U1" s="54" t="s">
+      <c r="U1" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="V1" s="54"/>
+      <c r="V1" s="60"/>
       <c r="W1" s="24"/>
       <c r="X1" s="24"/>
       <c r="Y1" s="25"/>
@@ -4384,10 +4397,10 @@
       <c r="B4" t="s">
         <v>547</v>
       </c>
-      <c r="C4" s="61">
+      <c r="C4" s="56">
         <v>212.7</v>
       </c>
-      <c r="D4" s="62" t="s">
+      <c r="D4" s="57" t="s">
         <v>514</v>
       </c>
       <c r="E4" t="s">
@@ -4446,10 +4459,10 @@
       <c r="B5" t="s">
         <v>548</v>
       </c>
-      <c r="C5" s="61">
+      <c r="C5" s="56">
         <v>212.7</v>
       </c>
-      <c r="D5" s="62" t="s">
+      <c r="D5" s="57" t="s">
         <v>514</v>
       </c>
       <c r="E5" t="s">
@@ -4508,10 +4521,10 @@
       <c r="B6" t="s">
         <v>549</v>
       </c>
-      <c r="C6" s="61">
+      <c r="C6" s="56">
         <v>212.8</v>
       </c>
-      <c r="D6" s="62" t="s">
+      <c r="D6" s="57" t="s">
         <v>514</v>
       </c>
       <c r="E6" t="s">
@@ -4567,10 +4580,10 @@
       <c r="B7" t="s">
         <v>550</v>
       </c>
-      <c r="C7" s="61">
+      <c r="C7" s="56">
         <v>212.7</v>
       </c>
-      <c r="D7" s="62" t="s">
+      <c r="D7" s="57" t="s">
         <v>514</v>
       </c>
       <c r="E7" t="s">
@@ -4626,10 +4639,10 @@
       <c r="B8" s="37" t="s">
         <v>551</v>
       </c>
-      <c r="C8" s="61">
+      <c r="C8" s="56">
         <v>212.2</v>
       </c>
-      <c r="D8" s="62" t="s">
+      <c r="D8" s="57" t="s">
         <v>514</v>
       </c>
       <c r="E8" t="s">
@@ -4685,10 +4698,10 @@
       <c r="B9" s="37" t="s">
         <v>552</v>
       </c>
-      <c r="C9" s="61">
+      <c r="C9" s="56">
         <v>212.4</v>
       </c>
-      <c r="D9" s="62" t="s">
+      <c r="D9" s="57" t="s">
         <v>514</v>
       </c>
       <c r="E9" t="s">
@@ -4744,10 +4757,10 @@
       <c r="B10" s="37" t="s">
         <v>553</v>
       </c>
-      <c r="C10" s="61">
+      <c r="C10" s="56">
         <v>212.6</v>
       </c>
-      <c r="D10" s="62" t="s">
+      <c r="D10" s="57" t="s">
         <v>514</v>
       </c>
       <c r="E10" t="s">
@@ -4803,10 +4816,10 @@
       <c r="B11" s="37" t="s">
         <v>554</v>
       </c>
-      <c r="C11" s="61">
+      <c r="C11" s="56">
         <v>212.9</v>
       </c>
-      <c r="D11" s="62" t="s">
+      <c r="D11" s="57" t="s">
         <v>514</v>
       </c>
       <c r="E11" t="s">
@@ -4862,10 +4875,10 @@
       <c r="B12" s="37" t="s">
         <v>555</v>
       </c>
-      <c r="C12" s="61">
+      <c r="C12" s="56">
         <v>213</v>
       </c>
-      <c r="D12" s="62" t="s">
+      <c r="D12" s="57" t="s">
         <v>514</v>
       </c>
       <c r="E12" t="s">
@@ -4921,10 +4934,10 @@
       <c r="B13" s="37" t="s">
         <v>556</v>
       </c>
-      <c r="C13" s="61">
+      <c r="C13" s="56">
         <v>213.2</v>
       </c>
-      <c r="D13" s="62" t="s">
+      <c r="D13" s="57" t="s">
         <v>514</v>
       </c>
       <c r="E13" t="s">
@@ -4980,10 +4993,10 @@
       <c r="B14" s="37" t="s">
         <v>557</v>
       </c>
-      <c r="C14" s="61">
+      <c r="C14" s="56">
         <v>213.4</v>
       </c>
-      <c r="D14" s="62" t="s">
+      <c r="D14" s="57" t="s">
         <v>514</v>
       </c>
       <c r="E14" t="s">
@@ -5039,10 +5052,10 @@
       <c r="B15" t="s">
         <v>546</v>
       </c>
-      <c r="C15" s="61">
+      <c r="C15" s="56">
         <v>213.65</v>
       </c>
-      <c r="D15" s="62" t="s">
+      <c r="D15" s="57" t="s">
         <v>514</v>
       </c>
       <c r="E15" t="s">
@@ -5098,10 +5111,10 @@
       <c r="B16" s="37" t="s">
         <v>558</v>
       </c>
-      <c r="C16" s="61">
+      <c r="C16" s="56">
         <v>213.75</v>
       </c>
-      <c r="D16" s="62" t="s">
+      <c r="D16" s="57" t="s">
         <v>514</v>
       </c>
       <c r="E16" t="s">
@@ -5157,10 +5170,10 @@
       <c r="B17" s="37" t="s">
         <v>559</v>
       </c>
-      <c r="C17" s="61">
+      <c r="C17" s="56">
         <v>142.5</v>
       </c>
-      <c r="D17" s="63" t="s">
+      <c r="D17" s="58" t="s">
         <v>515</v>
       </c>
       <c r="E17" t="s">
@@ -5216,10 +5229,10 @@
       <c r="B18" s="37" t="s">
         <v>560</v>
       </c>
-      <c r="C18" s="61">
+      <c r="C18" s="56">
         <v>150.80000000000001</v>
       </c>
-      <c r="D18" s="63" t="s">
+      <c r="D18" s="58" t="s">
         <v>515</v>
       </c>
       <c r="E18" t="s">
@@ -5275,10 +5288,10 @@
       <c r="B19" s="37" t="s">
         <v>561</v>
       </c>
-      <c r="C19" s="61">
+      <c r="C19" s="56">
         <v>164.2</v>
       </c>
-      <c r="D19" s="63" t="s">
+      <c r="D19" s="58" t="s">
         <v>515</v>
       </c>
       <c r="E19" t="s">
@@ -5334,10 +5347,10 @@
       <c r="B20" t="s">
         <v>562</v>
       </c>
-      <c r="C20" s="61">
+      <c r="C20" s="56">
         <v>168</v>
       </c>
-      <c r="D20" s="63" t="s">
+      <c r="D20" s="58" t="s">
         <v>515</v>
       </c>
       <c r="E20" t="s">
@@ -5393,10 +5406,10 @@
       <c r="B21" s="37" t="s">
         <v>563</v>
       </c>
-      <c r="C21" s="61">
+      <c r="C21" s="56">
         <v>206</v>
       </c>
-      <c r="D21" s="63" t="s">
+      <c r="D21" s="58" t="s">
         <v>515</v>
       </c>
       <c r="E21" t="s">
@@ -5452,10 +5465,10 @@
       <c r="B22" s="37" t="s">
         <v>564</v>
       </c>
-      <c r="C22" s="61">
+      <c r="C22" s="56">
         <v>215.1</v>
       </c>
-      <c r="D22" s="63" t="s">
+      <c r="D22" s="58" t="s">
         <v>515</v>
       </c>
       <c r="E22" t="s">
@@ -5511,10 +5524,10 @@
       <c r="B23" s="37" t="s">
         <v>565</v>
       </c>
-      <c r="C23" s="61">
+      <c r="C23" s="56">
         <v>11.2</v>
       </c>
-      <c r="D23" s="63" t="s">
+      <c r="D23" s="58" t="s">
         <v>516</v>
       </c>
       <c r="E23" t="s">
@@ -5573,10 +5586,10 @@
       <c r="B24" s="37" t="s">
         <v>566</v>
       </c>
-      <c r="C24" s="61">
+      <c r="C24" s="56">
         <v>69.5</v>
       </c>
-      <c r="D24" s="63" t="s">
+      <c r="D24" s="58" t="s">
         <v>516</v>
       </c>
       <c r="E24" t="s">
@@ -5635,10 +5648,10 @@
       <c r="B25" s="37" t="s">
         <v>567</v>
       </c>
-      <c r="C25" s="61">
+      <c r="C25" s="56">
         <v>22.4</v>
       </c>
-      <c r="D25" s="63" t="s">
+      <c r="D25" s="58" t="s">
         <v>517</v>
       </c>
       <c r="E25" t="s">
@@ -5697,10 +5710,10 @@
       <c r="B26" t="s">
         <v>568</v>
       </c>
-      <c r="C26" s="61">
+      <c r="C26" s="56">
         <v>32.799999999999997</v>
       </c>
-      <c r="D26" s="63" t="s">
+      <c r="D26" s="58" t="s">
         <v>517</v>
       </c>
       <c r="E26" t="s">
@@ -5759,10 +5772,10 @@
       <c r="B27" t="s">
         <v>569</v>
       </c>
-      <c r="C27" s="61">
+      <c r="C27" s="56">
         <v>42</v>
       </c>
-      <c r="D27" s="63" t="s">
+      <c r="D27" s="58" t="s">
         <v>517</v>
       </c>
       <c r="E27" t="s">
@@ -5821,10 +5834,10 @@
       <c r="B28" t="s">
         <v>570</v>
       </c>
-      <c r="C28" s="61">
+      <c r="C28" s="56">
         <v>50.7</v>
       </c>
-      <c r="D28" s="63" t="s">
+      <c r="D28" s="58" t="s">
         <v>517</v>
       </c>
       <c r="E28" t="s">
@@ -5883,10 +5896,10 @@
       <c r="B29" t="s">
         <v>571</v>
       </c>
-      <c r="C29" s="61">
+      <c r="C29" s="56">
         <v>62.6</v>
       </c>
-      <c r="D29" s="63" t="s">
+      <c r="D29" s="58" t="s">
         <v>517</v>
       </c>
       <c r="E29" t="s">
@@ -5945,10 +5958,10 @@
       <c r="B30" s="37" t="s">
         <v>572</v>
       </c>
-      <c r="C30" s="61">
+      <c r="C30" s="56">
         <v>72.400000000000006</v>
       </c>
-      <c r="D30" s="63" t="s">
+      <c r="D30" s="58" t="s">
         <v>517</v>
       </c>
       <c r="E30" t="s">
@@ -6007,10 +6020,10 @@
       <c r="B31" t="s">
         <v>573</v>
       </c>
-      <c r="C31" s="61">
+      <c r="C31" s="56">
         <v>81.2</v>
       </c>
-      <c r="D31" s="63" t="s">
+      <c r="D31" s="58" t="s">
         <v>517</v>
       </c>
       <c r="E31" t="s">
@@ -6069,10 +6082,10 @@
       <c r="B32" t="s">
         <v>574</v>
       </c>
-      <c r="C32" s="61">
+      <c r="C32" s="56">
         <v>91.6</v>
       </c>
-      <c r="D32" s="63" t="s">
+      <c r="D32" s="58" t="s">
         <v>517</v>
       </c>
       <c r="E32" t="s">
@@ -6131,10 +6144,10 @@
       <c r="B33" t="s">
         <v>575</v>
       </c>
-      <c r="C33" s="61">
+      <c r="C33" s="56">
         <v>100.8</v>
       </c>
-      <c r="D33" s="63" t="s">
+      <c r="D33" s="58" t="s">
         <v>517</v>
       </c>
       <c r="E33" t="s">
@@ -6193,10 +6206,10 @@
       <c r="B34" s="37" t="s">
         <v>576</v>
       </c>
-      <c r="C34" s="61">
+      <c r="C34" s="56">
         <v>110.1</v>
       </c>
-      <c r="D34" s="63" t="s">
+      <c r="D34" s="58" t="s">
         <v>517</v>
       </c>
       <c r="E34" t="s">
@@ -6255,10 +6268,10 @@
       <c r="B35" s="37" t="s">
         <v>577</v>
       </c>
-      <c r="C35" s="64">
+      <c r="C35" s="59">
         <v>121.6</v>
       </c>
-      <c r="D35" s="63" t="s">
+      <c r="D35" s="58" t="s">
         <v>517</v>
       </c>
       <c r="E35" t="s">
@@ -6317,10 +6330,10 @@
       <c r="B36" s="37" t="s">
         <v>578</v>
       </c>
-      <c r="C36" s="64">
+      <c r="C36" s="59">
         <v>131.9</v>
       </c>
-      <c r="D36" s="63" t="s">
+      <c r="D36" s="58" t="s">
         <v>517</v>
       </c>
       <c r="E36" t="s">
@@ -6379,10 +6392,10 @@
       <c r="B37" s="37" t="s">
         <v>579</v>
       </c>
-      <c r="C37" s="64">
+      <c r="C37" s="59">
         <v>143</v>
       </c>
-      <c r="D37" s="63" t="s">
+      <c r="D37" s="58" t="s">
         <v>517</v>
       </c>
       <c r="E37" t="s">
@@ -6441,10 +6454,10 @@
       <c r="B38" s="37" t="s">
         <v>580</v>
       </c>
-      <c r="C38" s="64">
+      <c r="C38" s="59">
         <v>154.30000000000001</v>
       </c>
-      <c r="D38" s="63" t="s">
+      <c r="D38" s="58" t="s">
         <v>517</v>
       </c>
       <c r="E38" t="s">
@@ -6503,10 +6516,10 @@
       <c r="B39" s="37" t="s">
         <v>581</v>
       </c>
-      <c r="C39" s="64">
+      <c r="C39" s="59">
         <v>162.30000000000001</v>
       </c>
-      <c r="D39" s="63" t="s">
+      <c r="D39" s="58" t="s">
         <v>517</v>
       </c>
       <c r="E39" t="s">
@@ -6565,10 +6578,10 @@
       <c r="B40" s="37" t="s">
         <v>582</v>
       </c>
-      <c r="C40" s="64">
+      <c r="C40" s="59">
         <v>174.9</v>
       </c>
-      <c r="D40" s="63" t="s">
+      <c r="D40" s="58" t="s">
         <v>517</v>
       </c>
       <c r="E40" t="s">
@@ -6627,10 +6640,10 @@
       <c r="B41" s="37" t="s">
         <v>583</v>
       </c>
-      <c r="C41" s="64">
+      <c r="C41" s="59">
         <v>0.2</v>
       </c>
-      <c r="D41" s="63" t="s">
+      <c r="D41" s="58" t="s">
         <v>518</v>
       </c>
       <c r="E41" t="s">
@@ -6689,10 +6702,10 @@
       <c r="B42" s="37" t="s">
         <v>584</v>
       </c>
-      <c r="C42" s="64">
+      <c r="C42" s="59">
         <v>0.4</v>
       </c>
-      <c r="D42" s="63" t="s">
+      <c r="D42" s="58" t="s">
         <v>518</v>
       </c>
       <c r="E42" t="s">
@@ -6751,10 +6764,10 @@
       <c r="B43" s="37" t="s">
         <v>585</v>
       </c>
-      <c r="C43" s="64">
+      <c r="C43" s="59">
         <v>0.6</v>
       </c>
-      <c r="D43" s="63" t="s">
+      <c r="D43" s="58" t="s">
         <v>518</v>
       </c>
       <c r="E43" t="s">
@@ -6813,10 +6826,10 @@
       <c r="B44" t="s">
         <v>586</v>
       </c>
-      <c r="C44" s="64">
+      <c r="C44" s="59">
         <v>0.7</v>
       </c>
-      <c r="D44" s="63" t="s">
+      <c r="D44" s="58" t="s">
         <v>518</v>
       </c>
       <c r="E44" t="s">
@@ -6875,10 +6888,10 @@
       <c r="B45" t="s">
         <v>587</v>
       </c>
-      <c r="C45" s="64">
+      <c r="C45" s="59">
         <v>0.8</v>
       </c>
-      <c r="D45" s="63" t="s">
+      <c r="D45" s="58" t="s">
         <v>518</v>
       </c>
       <c r="E45" t="s">
@@ -6937,10 +6950,10 @@
       <c r="B46" s="37" t="s">
         <v>588</v>
       </c>
-      <c r="C46" s="64">
+      <c r="C46" s="59">
         <v>1</v>
       </c>
-      <c r="D46" s="63" t="s">
+      <c r="D46" s="58" t="s">
         <v>518</v>
       </c>
       <c r="E46" t="s">
@@ -6999,10 +7012,10 @@
       <c r="B47" s="37" t="s">
         <v>589</v>
       </c>
-      <c r="C47" s="64">
+      <c r="C47" s="59">
         <v>1.1000000000000001</v>
       </c>
-      <c r="D47" s="63" t="s">
+      <c r="D47" s="58" t="s">
         <v>518</v>
       </c>
       <c r="E47" t="s">
@@ -7061,10 +7074,10 @@
       <c r="B48" s="37" t="s">
         <v>590</v>
       </c>
-      <c r="C48" s="64">
+      <c r="C48" s="59">
         <v>1.2</v>
       </c>
-      <c r="D48" s="63" t="s">
+      <c r="D48" s="58" t="s">
         <v>518</v>
       </c>
       <c r="E48" t="s">
@@ -7123,10 +7136,10 @@
       <c r="B49" s="37" t="s">
         <v>591</v>
       </c>
-      <c r="C49" s="64">
+      <c r="C49" s="59">
         <v>1.35</v>
       </c>
-      <c r="D49" s="63" t="s">
+      <c r="D49" s="58" t="s">
         <v>518</v>
       </c>
       <c r="E49" t="s">
@@ -7185,10 +7198,10 @@
       <c r="B50" s="37" t="s">
         <v>592</v>
       </c>
-      <c r="C50" s="64">
+      <c r="C50" s="59">
         <v>1.4</v>
       </c>
-      <c r="D50" s="63" t="s">
+      <c r="D50" s="58" t="s">
         <v>518</v>
       </c>
       <c r="E50" t="s">
@@ -7247,10 +7260,10 @@
       <c r="B51" s="37" t="s">
         <v>593</v>
       </c>
-      <c r="C51" s="64">
+      <c r="C51" s="59">
         <v>0</v>
       </c>
-      <c r="D51" s="63" t="s">
+      <c r="D51" s="58" t="s">
         <v>519</v>
       </c>
       <c r="E51" t="s">
@@ -7309,10 +7322,10 @@
       <c r="B52" s="37" t="s">
         <v>594</v>
       </c>
-      <c r="C52" s="64">
+      <c r="C52" s="59">
         <v>0.1</v>
       </c>
-      <c r="D52" s="63" t="s">
+      <c r="D52" s="58" t="s">
         <v>519</v>
       </c>
       <c r="E52" t="s">
@@ -7371,10 +7384,10 @@
       <c r="B53" s="37" t="s">
         <v>595</v>
       </c>
-      <c r="C53" s="64">
+      <c r="C53" s="59">
         <v>0.3</v>
       </c>
-      <c r="D53" s="63" t="s">
+      <c r="D53" s="58" t="s">
         <v>519</v>
       </c>
       <c r="E53" t="s">
@@ -7433,10 +7446,10 @@
       <c r="B54" s="37" t="s">
         <v>596</v>
       </c>
-      <c r="C54" s="64">
+      <c r="C54" s="59">
         <v>0.6</v>
       </c>
-      <c r="D54" s="63" t="s">
+      <c r="D54" s="58" t="s">
         <v>519</v>
       </c>
       <c r="E54" t="s">
@@ -7495,10 +7508,10 @@
       <c r="B55" t="s">
         <v>597</v>
       </c>
-      <c r="C55" s="64">
+      <c r="C55" s="59">
         <v>0.75</v>
       </c>
-      <c r="D55" s="63" t="s">
+      <c r="D55" s="58" t="s">
         <v>519</v>
       </c>
       <c r="E55" t="s">
@@ -7557,10 +7570,10 @@
       <c r="B56" s="37" t="s">
         <v>598</v>
       </c>
-      <c r="C56" s="64">
+      <c r="C56" s="59">
         <v>0.85</v>
       </c>
-      <c r="D56" s="63" t="s">
+      <c r="D56" s="58" t="s">
         <v>519</v>
       </c>
       <c r="E56" t="s">
@@ -7616,13 +7629,13 @@
       </c>
     </row>
     <row r="57" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B57" s="59" t="s">
+      <c r="B57" s="54" t="s">
         <v>599</v>
       </c>
-      <c r="C57" s="64">
+      <c r="C57" s="59">
         <v>2.2999999999999998</v>
       </c>
-      <c r="D57" s="63" t="s">
+      <c r="D57" s="58" t="s">
         <v>520</v>
       </c>
       <c r="E57" t="s">
@@ -7678,10 +7691,10 @@
       <c r="B58" s="37" t="s">
         <v>600</v>
       </c>
-      <c r="C58" s="64">
+      <c r="C58" s="59">
         <v>2.1</v>
       </c>
-      <c r="D58" s="63" t="s">
+      <c r="D58" s="58" t="s">
         <v>520</v>
       </c>
       <c r="E58" t="s">
@@ -7737,10 +7750,10 @@
       <c r="B59" s="37" t="s">
         <v>601</v>
       </c>
-      <c r="C59" s="64">
+      <c r="C59" s="59">
         <v>1.9</v>
       </c>
-      <c r="D59" s="63" t="s">
+      <c r="D59" s="58" t="s">
         <v>520</v>
       </c>
       <c r="E59" t="s">
@@ -7796,10 +7809,10 @@
       <c r="B60" s="37" t="s">
         <v>602</v>
       </c>
-      <c r="C60" s="64">
+      <c r="C60" s="59">
         <v>0.3</v>
       </c>
-      <c r="D60" s="63" t="s">
+      <c r="D60" s="58" t="s">
         <v>520</v>
       </c>
       <c r="E60" t="s">
@@ -7852,13 +7865,13 @@
       </c>
     </row>
     <row r="61" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B61" s="59" t="s">
+      <c r="B61" s="54" t="s">
         <v>603</v>
       </c>
-      <c r="C61" s="64">
+      <c r="C61" s="59">
         <v>1.2</v>
       </c>
-      <c r="D61" s="63" t="s">
+      <c r="D61" s="58" t="s">
         <v>520</v>
       </c>
       <c r="E61" t="s">
@@ -7914,10 +7927,10 @@
       <c r="B62" s="37" t="s">
         <v>604</v>
       </c>
-      <c r="C62" s="64">
+      <c r="C62" s="59">
         <v>2.4</v>
       </c>
-      <c r="D62" s="63" t="s">
+      <c r="D62" s="58" t="s">
         <v>520</v>
       </c>
       <c r="E62" t="s">
@@ -7970,13 +7983,13 @@
       </c>
     </row>
     <row r="63" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B63" s="60" t="s">
+      <c r="B63" s="55" t="s">
         <v>605</v>
       </c>
-      <c r="C63" s="64">
+      <c r="C63" s="59">
         <v>1.2</v>
       </c>
-      <c r="D63" s="63" t="s">
+      <c r="D63" s="58" t="s">
         <v>520</v>
       </c>
       <c r="E63" t="s">
@@ -8029,13 +8042,13 @@
       </c>
     </row>
     <row r="64" spans="2:27" ht="17" x14ac:dyDescent="0.2">
-      <c r="B64" s="60" t="s">
+      <c r="B64" s="55" t="s">
         <v>606</v>
       </c>
-      <c r="C64" s="64">
+      <c r="C64" s="59">
         <v>0.3</v>
       </c>
-      <c r="D64" s="63" t="s">
+      <c r="D64" s="58" t="s">
         <v>520</v>
       </c>
       <c r="E64" t="s">
@@ -8091,10 +8104,10 @@
       <c r="B65" t="s">
         <v>607</v>
       </c>
-      <c r="C65" s="64">
+      <c r="C65" s="59">
         <v>1.9</v>
       </c>
-      <c r="D65" s="63" t="s">
+      <c r="D65" s="58" t="s">
         <v>520</v>
       </c>
       <c r="E65" t="s">
@@ -8150,10 +8163,10 @@
       <c r="B66" t="s">
         <v>608</v>
       </c>
-      <c r="C66" s="64">
+      <c r="C66" s="59">
         <v>2.4</v>
       </c>
-      <c r="D66" s="63" t="s">
+      <c r="D66" s="58" t="s">
         <v>520</v>
       </c>
       <c r="E66" t="s">
@@ -8709,22 +8722,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="62" t="s">
         <v>225</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
       <c r="E1" s="14" t="s">
         <v>226</v>
       </c>
       <c r="F1" s="14"/>
       <c r="G1" s="14"/>
-      <c r="H1" s="56" t="s">
+      <c r="H1" s="63" t="s">
         <v>227</v>
       </c>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
       <c r="K1" s="5" t="s">
         <v>228</v>
       </c>
@@ -8732,18 +8745,18 @@
       <c r="M1" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="N1" s="57" t="s">
+      <c r="N1" s="64" t="s">
         <v>260</v>
       </c>
-      <c r="O1" s="57"/>
-      <c r="P1" s="57"/>
-      <c r="Q1" s="57"/>
-      <c r="R1" s="57"/>
-      <c r="S1" s="55" t="s">
+      <c r="O1" s="64"/>
+      <c r="P1" s="64"/>
+      <c r="Q1" s="64"/>
+      <c r="R1" s="64"/>
+      <c r="S1" s="62" t="s">
         <v>142</v>
       </c>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
       <c r="V1" s="19" t="s">
         <v>237</v>
       </c>

</xml_diff>